<commit_message>
Update and rename EASMailboxMSS.fsh to AsMailboxMSSExtension.fsh 5310f5fd808d925e3e78e1d041ad89e9c2d289a0
</commit_message>
<xml_diff>
--- a/ig/feature-good-practices-interop/StructureDefinition-as-ext-mailbox-mss.xlsx
+++ b/ig/feature-good-practices-interop/StructureDefinition-as-ext-mailbox-mss.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$63</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2067" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2098" uniqueCount="255">
   <si>
     <t>Property</t>
   </si>
@@ -39,13 +39,13 @@
     <t>Name</t>
   </si>
   <si>
-    <t>EASMailboxMSS</t>
+    <t>AsMailboxMSSExtension</t>
   </si>
   <si>
     <t>Title</t>
   </si>
   <si>
-    <t>EAS Mailbox MSS</t>
+    <t>AS Mailbox MSS Extension</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-04-13T08:12:13+00:00</t>
+    <t>2023-04-13T08:22:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -421,13 +421,14 @@
 PER pour une BAL personnelle, rattachée à une personne physique</t>
   </si>
   <si>
-    <t>required</t>
-  </si>
-  <si>
     <t>Type de  boîte aux lettre MSS</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J139-TypeBAL-RASS/FHIR/JDV-J139-TypeBAL-RASS</t>
+    <t xml:space="preserve">type:$this}
+</t>
+  </si>
+  <si>
+    <t>closed</t>
   </si>
   <si>
     <t>Extension.extension:type.value[x].id</t>
@@ -629,6 +630,18 @@
   </si>
   <si>
     <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
+    <t>Extension.extension:type.value[x]:valueCodeableConcept</t>
+  </si>
+  <si>
+    <t>valueCodeableConcept</t>
+  </si>
+  <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J139-TypeBAL-RASS/FHIR/JDV-J139-TypeBAL-RASS</t>
   </si>
   <si>
     <t>Extension.extension:description</t>
@@ -1121,12 +1134,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK62"/>
+  <dimension ref="A1:AK63"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="51.65625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="54.2421875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="46.94140625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="12.66015625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="22.25390625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="12.64453125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.9453125" customWidth="true" bestFit="true"/>
@@ -2582,28 +2595,26 @@
         <v>76</v>
       </c>
       <c r="X14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y14" t="s" s="2">
         <v>130</v>
       </c>
-      <c r="Y14" t="s" s="2">
+      <c r="Z14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB14" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="Z14" t="s" s="2">
+      <c r="AC14" s="2"/>
+      <c r="AD14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE14" t="s" s="2">
         <v>132</v>
-      </c>
-      <c r="AA14" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB14" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC14" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AD14" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE14" t="s" s="2">
-        <v>76</v>
       </c>
       <c r="AF14" t="s" s="2">
         <v>120</v>
@@ -3792,7 +3803,7 @@
         <v>199</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="C26" t="s" s="2">
         <v>200</v>
@@ -3808,7 +3819,7 @@
         <v>82</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>76</v>
@@ -3817,13 +3828,13 @@
         <v>76</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -3850,13 +3861,11 @@
         <v>76</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y26" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="Y26" s="2"/>
       <c r="Z26" t="s" s="2">
-        <v>76</v>
+        <v>202</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>76</v>
@@ -3874,32 +3883,34 @@
         <v>76</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="C27" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="C27" t="s" s="2">
+        <v>204</v>
+      </c>
       <c r="D27" t="s" s="2">
         <v>76</v>
       </c>
@@ -3911,7 +3922,7 @@
         <v>82</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>76</v>
@@ -3920,13 +3931,13 @@
         <v>76</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3977,30 +3988,30 @@
         <v>76</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI27" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4011,7 +4022,7 @@
         <v>77</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>76</v>
@@ -4023,13 +4034,13 @@
         <v>76</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4068,42 +4079,42 @@
         <v>76</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC28" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD28" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE28" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI28" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4111,10 +4122,10 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>76</v>
@@ -4126,24 +4137,22 @@
         <v>76</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" t="s" s="2">
-        <v>200</v>
+        <v>76</v>
       </c>
       <c r="S29" t="s" s="2">
         <v>76</v>
@@ -4173,42 +4182,42 @@
         <v>76</v>
       </c>
       <c r="AB29" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AC29" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AD29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE29" t="s" s="2">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AG29" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI29" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4216,7 +4225,7 @@
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G30" t="s" s="2">
         <v>82</v>
@@ -4231,22 +4240,24 @@
         <v>76</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>205</v>
+        <v>112</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q30" s="2"/>
       <c r="R30" t="s" s="2">
-        <v>76</v>
+        <v>204</v>
       </c>
       <c r="S30" t="s" s="2">
         <v>76</v>
@@ -4288,19 +4299,19 @@
         <v>76</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG30" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH30" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>99</v>
@@ -4308,14 +4319,12 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="C31" t="s" s="2">
-        <v>207</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
         <v>76</v>
       </c>
@@ -4327,7 +4336,7 @@
         <v>82</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>76</v>
@@ -4336,13 +4345,13 @@
         <v>76</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>28</v>
+        <v>209</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4393,32 +4402,34 @@
         <v>76</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="C32" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="C32" t="s" s="2">
+        <v>211</v>
+      </c>
       <c r="D32" t="s" s="2">
         <v>76</v>
       </c>
@@ -4430,7 +4441,7 @@
         <v>82</v>
       </c>
       <c r="H32" t="s" s="2">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="I32" t="s" s="2">
         <v>76</v>
@@ -4439,13 +4450,13 @@
         <v>76</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4496,30 +4507,30 @@
         <v>76</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4530,7 +4541,7 @@
         <v>77</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>76</v>
@@ -4542,13 +4553,13 @@
         <v>76</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -4587,42 +4598,42 @@
         <v>76</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC33" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD33" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI33" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4630,10 +4641,10 @@
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>76</v>
@@ -4645,24 +4656,22 @@
         <v>76</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q34" s="2"/>
       <c r="R34" t="s" s="2">
-        <v>207</v>
+        <v>76</v>
       </c>
       <c r="S34" t="s" s="2">
         <v>76</v>
@@ -4692,42 +4701,42 @@
         <v>76</v>
       </c>
       <c r="AB34" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AC34" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AD34" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE34" t="s" s="2">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4735,7 +4744,7 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>82</v>
@@ -4750,22 +4759,24 @@
         <v>76</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>212</v>
+        <v>112</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="N35" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N35" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q35" s="2"/>
       <c r="R35" t="s" s="2">
-        <v>76</v>
+        <v>211</v>
       </c>
       <c r="S35" t="s" s="2">
         <v>76</v>
@@ -4807,19 +4818,19 @@
         <v>76</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH35" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI35" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK35" t="s" s="2">
         <v>99</v>
@@ -4827,14 +4838,12 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>214</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
         <v>76</v>
       </c>
@@ -4846,7 +4855,7 @@
         <v>82</v>
       </c>
       <c r="H36" t="s" s="2">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="I36" t="s" s="2">
         <v>76</v>
@@ -4855,13 +4864,13 @@
         <v>76</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>28</v>
+        <v>216</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -4912,32 +4921,34 @@
         <v>76</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="C37" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="C37" t="s" s="2">
+        <v>218</v>
+      </c>
       <c r="D37" t="s" s="2">
         <v>76</v>
       </c>
@@ -4949,7 +4960,7 @@
         <v>82</v>
       </c>
       <c r="H37" t="s" s="2">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="I37" t="s" s="2">
         <v>76</v>
@@ -4958,13 +4969,13 @@
         <v>76</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5015,30 +5026,30 @@
         <v>76</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI37" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5049,7 +5060,7 @@
         <v>77</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>76</v>
@@ -5061,13 +5072,13 @@
         <v>76</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5106,42 +5117,42 @@
         <v>76</v>
       </c>
       <c r="AB38" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC38" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD38" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE38" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5149,10 +5160,10 @@
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>76</v>
@@ -5164,24 +5175,22 @@
         <v>76</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q39" s="2"/>
       <c r="R39" t="s" s="2">
-        <v>214</v>
+        <v>76</v>
       </c>
       <c r="S39" t="s" s="2">
         <v>76</v>
@@ -5211,42 +5220,42 @@
         <v>76</v>
       </c>
       <c r="AB39" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AC39" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AD39" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE39" t="s" s="2">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AG39" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5254,7 +5263,7 @@
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G40" t="s" s="2">
         <v>82</v>
@@ -5269,22 +5278,24 @@
         <v>76</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>219</v>
+        <v>112</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="N40" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q40" s="2"/>
       <c r="R40" t="s" s="2">
-        <v>76</v>
+        <v>218</v>
       </c>
       <c r="S40" t="s" s="2">
         <v>76</v>
@@ -5326,19 +5337,19 @@
         <v>76</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG40" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH40" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI40" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>99</v>
@@ -5346,14 +5357,12 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="C41" t="s" s="2">
-        <v>221</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
         <v>76</v>
       </c>
@@ -5365,7 +5374,7 @@
         <v>82</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>76</v>
@@ -5374,13 +5383,13 @@
         <v>76</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>28</v>
+        <v>223</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -5431,32 +5440,34 @@
         <v>76</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="C42" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="C42" t="s" s="2">
+        <v>225</v>
+      </c>
       <c r="D42" t="s" s="2">
         <v>76</v>
       </c>
@@ -5468,7 +5479,7 @@
         <v>82</v>
       </c>
       <c r="H42" t="s" s="2">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="I42" t="s" s="2">
         <v>76</v>
@@ -5477,13 +5488,13 @@
         <v>76</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -5534,30 +5545,30 @@
         <v>76</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI42" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -5568,7 +5579,7 @@
         <v>77</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>76</v>
@@ -5580,13 +5591,13 @@
         <v>76</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -5625,42 +5636,42 @@
         <v>76</v>
       </c>
       <c r="AB43" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC43" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD43" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE43" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI43" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -5668,10 +5679,10 @@
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>76</v>
@@ -5683,24 +5694,22 @@
         <v>76</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q44" s="2"/>
       <c r="R44" t="s" s="2">
-        <v>221</v>
+        <v>76</v>
       </c>
       <c r="S44" t="s" s="2">
         <v>76</v>
@@ -5730,42 +5739,42 @@
         <v>76</v>
       </c>
       <c r="AB44" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AC44" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AD44" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE44" t="s" s="2">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AG44" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -5773,7 +5782,7 @@
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G45" t="s" s="2">
         <v>82</v>
@@ -5788,22 +5797,24 @@
         <v>76</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>226</v>
+        <v>112</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="N45" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q45" s="2"/>
       <c r="R45" t="s" s="2">
-        <v>76</v>
+        <v>225</v>
       </c>
       <c r="S45" t="s" s="2">
         <v>76</v>
@@ -5845,19 +5856,19 @@
         <v>76</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG45" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH45" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK45" t="s" s="2">
         <v>99</v>
@@ -5865,14 +5876,12 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="C46" t="s" s="2">
-        <v>228</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
         <v>76</v>
       </c>
@@ -5884,7 +5893,7 @@
         <v>82</v>
       </c>
       <c r="H46" t="s" s="2">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="I46" t="s" s="2">
         <v>76</v>
@@ -5893,13 +5902,13 @@
         <v>76</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>28</v>
+        <v>230</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -5950,32 +5959,34 @@
         <v>76</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="C47" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="C47" t="s" s="2">
+        <v>232</v>
+      </c>
       <c r="D47" t="s" s="2">
         <v>76</v>
       </c>
@@ -5987,7 +5998,7 @@
         <v>82</v>
       </c>
       <c r="H47" t="s" s="2">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="I47" t="s" s="2">
         <v>76</v>
@@ -5996,13 +6007,13 @@
         <v>76</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -6053,30 +6064,30 @@
         <v>76</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ47" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6087,7 +6098,7 @@
         <v>77</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>76</v>
@@ -6099,13 +6110,13 @@
         <v>76</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -6144,42 +6155,42 @@
         <v>76</v>
       </c>
       <c r="AB48" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC48" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD48" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE48" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI48" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ48" t="s" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6187,10 +6198,10 @@
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>76</v>
@@ -6202,24 +6213,22 @@
         <v>76</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q49" s="2"/>
       <c r="R49" t="s" s="2">
-        <v>228</v>
+        <v>76</v>
       </c>
       <c r="S49" t="s" s="2">
         <v>76</v>
@@ -6249,42 +6258,42 @@
         <v>76</v>
       </c>
       <c r="AB49" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AC49" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AD49" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE49" t="s" s="2">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AG49" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH49" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI49" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK49" t="s" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -6292,7 +6301,7 @@
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G50" t="s" s="2">
         <v>82</v>
@@ -6307,16 +6316,16 @@
         <v>76</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>184</v>
+        <v>111</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>233</v>
+        <v>112</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>234</v>
+        <v>114</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
@@ -6324,7 +6333,7 @@
       </c>
       <c r="Q50" s="2"/>
       <c r="R50" t="s" s="2">
-        <v>76</v>
+        <v>232</v>
       </c>
       <c r="S50" t="s" s="2">
         <v>76</v>
@@ -6366,19 +6375,19 @@
         <v>76</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG50" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH50" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI50" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ50" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK50" t="s" s="2">
         <v>99</v>
@@ -6386,14 +6395,12 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="C51" t="s" s="2">
-        <v>236</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
         <v>76</v>
       </c>
@@ -6405,7 +6412,7 @@
         <v>82</v>
       </c>
       <c r="H51" t="s" s="2">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="I51" t="s" s="2">
         <v>76</v>
@@ -6414,15 +6421,17 @@
         <v>76</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>90</v>
+        <v>184</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>28</v>
+        <v>237</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="N51" s="2"/>
+        <v>119</v>
+      </c>
+      <c r="N51" t="s" s="2">
+        <v>238</v>
+      </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
         <v>76</v>
@@ -6471,32 +6480,34 @@
         <v>76</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI51" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="C52" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="C52" t="s" s="2">
+        <v>240</v>
+      </c>
       <c r="D52" t="s" s="2">
         <v>76</v>
       </c>
@@ -6508,7 +6519,7 @@
         <v>82</v>
       </c>
       <c r="H52" t="s" s="2">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="I52" t="s" s="2">
         <v>76</v>
@@ -6517,13 +6528,13 @@
         <v>76</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -6574,30 +6585,30 @@
         <v>76</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH52" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI52" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ52" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -6608,7 +6619,7 @@
         <v>77</v>
       </c>
       <c r="G53" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H53" t="s" s="2">
         <v>76</v>
@@ -6620,13 +6631,13 @@
         <v>76</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -6665,42 +6676,42 @@
         <v>76</v>
       </c>
       <c r="AB53" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC53" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD53" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE53" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH53" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI53" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ53" t="s" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -6708,10 +6719,10 @@
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>76</v>
@@ -6723,24 +6734,22 @@
         <v>76</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N54" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N54" s="2"/>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q54" s="2"/>
       <c r="R54" t="s" s="2">
-        <v>236</v>
+        <v>76</v>
       </c>
       <c r="S54" t="s" s="2">
         <v>76</v>
@@ -6770,42 +6779,42 @@
         <v>76</v>
       </c>
       <c r="AB54" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AC54" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AD54" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE54" t="s" s="2">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AG54" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI54" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ54" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -6813,7 +6822,7 @@
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G55" t="s" s="2">
         <v>82</v>
@@ -6828,16 +6837,16 @@
         <v>76</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>184</v>
+        <v>111</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>241</v>
+        <v>112</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>242</v>
+        <v>114</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
@@ -6845,7 +6854,7 @@
       </c>
       <c r="Q55" s="2"/>
       <c r="R55" t="s" s="2">
-        <v>76</v>
+        <v>240</v>
       </c>
       <c r="S55" t="s" s="2">
         <v>76</v>
@@ -6887,19 +6896,19 @@
         <v>76</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG55" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH55" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI55" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ55" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK55" t="s" s="2">
         <v>99</v>
@@ -6907,14 +6916,12 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="C56" t="s" s="2">
-        <v>244</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
         <v>76</v>
       </c>
@@ -6923,10 +6930,10 @@
         <v>77</v>
       </c>
       <c r="G56" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H56" t="s" s="2">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="I56" t="s" s="2">
         <v>76</v>
@@ -6935,15 +6942,17 @@
         <v>76</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>90</v>
+        <v>184</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>28</v>
+        <v>245</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="N56" s="2"/>
+        <v>119</v>
+      </c>
+      <c r="N56" t="s" s="2">
+        <v>246</v>
+      </c>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
         <v>76</v>
@@ -6992,32 +7001,34 @@
         <v>76</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH56" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI56" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ56" t="s" s="2">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="C57" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="C57" t="s" s="2">
+        <v>248</v>
+      </c>
       <c r="D57" t="s" s="2">
         <v>76</v>
       </c>
@@ -7026,7 +7037,7 @@
         <v>77</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>76</v>
@@ -7038,13 +7049,13 @@
         <v>76</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -7095,30 +7106,30 @@
         <v>76</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH57" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI57" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK57" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -7129,7 +7140,7 @@
         <v>77</v>
       </c>
       <c r="G58" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H58" t="s" s="2">
         <v>76</v>
@@ -7141,13 +7152,13 @@
         <v>76</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -7186,42 +7197,42 @@
         <v>76</v>
       </c>
       <c r="AB58" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC58" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD58" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE58" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH58" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI58" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AK58" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -7229,10 +7240,10 @@
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G59" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="H59" t="s" s="2">
         <v>76</v>
@@ -7244,24 +7255,22 @@
         <v>76</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N59" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N59" s="2"/>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q59" s="2"/>
       <c r="R59" t="s" s="2">
-        <v>244</v>
+        <v>76</v>
       </c>
       <c r="S59" t="s" s="2">
         <v>76</v>
@@ -7291,42 +7300,42 @@
         <v>76</v>
       </c>
       <c r="AB59" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AC59" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AD59" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE59" t="s" s="2">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AG59" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH59" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI59" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -7334,7 +7343,7 @@
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G60" t="s" s="2">
         <v>82</v>
@@ -7349,22 +7358,24 @@
         <v>76</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>249</v>
+        <v>111</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="N60" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N60" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q60" s="2"/>
       <c r="R60" t="s" s="2">
-        <v>76</v>
+        <v>248</v>
       </c>
       <c r="S60" t="s" s="2">
         <v>76</v>
@@ -7406,19 +7417,19 @@
         <v>76</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG60" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH60" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI60" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ60" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK60" t="s" s="2">
         <v>99</v>
@@ -7426,10 +7437,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>115</v>
+        <v>252</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -7437,7 +7448,7 @@
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G61" t="s" s="2">
         <v>82</v>
@@ -7452,24 +7463,22 @@
         <v>76</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>111</v>
+        <v>253</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="N61" s="2"/>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q61" s="2"/>
       <c r="R61" t="s" s="2">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="S61" t="s" s="2">
         <v>76</v>
@@ -7511,19 +7520,19 @@
         <v>76</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="AG61" t="s" s="2">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="AH61" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI61" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ61" t="s" s="2">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="AK61" t="s" s="2">
         <v>99</v>
@@ -7531,10 +7540,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -7542,10 +7551,10 @@
       </c>
       <c r="E62" s="2"/>
       <c r="F62" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G62" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H62" t="s" s="2">
         <v>76</v>
@@ -7557,22 +7566,24 @@
         <v>76</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>250</v>
+        <v>111</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="N62" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N62" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q62" s="2"/>
       <c r="R62" t="s" s="2">
-        <v>76</v>
+        <v>3</v>
       </c>
       <c r="S62" t="s" s="2">
         <v>76</v>
@@ -7614,26 +7625,129 @@
         <v>76</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="AG62" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="AH62" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AI62" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ62" t="s" s="2">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="AK62" t="s" s="2">
         <v>99</v>
       </c>
     </row>
+    <row r="63" hidden="true">
+      <c r="A63" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="B63" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="C63" s="2"/>
+      <c r="D63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E63" s="2"/>
+      <c r="F63" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G63" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K63" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="L63" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="M63" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="N63" s="2"/>
+      <c r="O63" s="2"/>
+      <c r="P63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q63" s="2"/>
+      <c r="R63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF63" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AG63" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH63" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI63" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ63" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="AK63" t="s" s="2">
+        <v>99</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AK62">
+  <autoFilter ref="A1:AK63">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -7643,7 +7757,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI61">
+  <conditionalFormatting sqref="A2:AI62">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>